<commit_message>
chore(stoicisme-lecon): livrables auto 2026-10-01
</commit_message>
<xml_diff>
--- a/livrables/documents/2026-08-09_Les 14 Jobs.xlsx
+++ b/livrables/documents/2026-08-09_Les 14 Jobs.xlsx
@@ -762,7 +762,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -789,7 +789,7 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(controle-livrables): livrables auto 2026-10-04
</commit_message>
<xml_diff>
--- a/livrables/documents/2026-08-09_Les 14 Jobs.xlsx
+++ b/livrables/documents/2026-08-09_Les 14 Jobs.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>—</t>
         </is>
       </c>
     </row>

</xml_diff>